<commit_message>
UK daily ratings for 2026-04-16
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-04-16.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-04-16.xlsx
@@ -528,17 +528,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Enricher (IRE)</t>
+          <t>Pilu (IRE)</t>
         </is>
       </c>
       <c r="I2" t="n">
         <v>3</v>
       </c>
       <c r="J2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="K2" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -584,17 +584,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Pilu (IRE)</t>
+          <t>Reciprocated</t>
         </is>
       </c>
       <c r="I3" t="n">
         <v>3</v>
       </c>
       <c r="J3" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="K3" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -640,17 +640,17 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Reciprocated</t>
+          <t>Enricher (IRE)</t>
         </is>
       </c>
       <c r="I4" t="n">
         <v>3</v>
       </c>
       <c r="J4" t="n">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="K4" t="n">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -2902,7 +2902,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Hawk Mountain (IRE)</t>
+          <t>Hankelow (IRE)</t>
         </is>
       </c>
       <c r="I42" t="n">
@@ -2912,7 +2912,7 @@
         <v>128</v>
       </c>
       <c r="K42" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="n">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Hankelow (IRE)</t>
+          <t>Hawk Mountain (IRE)</t>
         </is>
       </c>
       <c r="I43" t="n">
@@ -2968,7 +2968,7 @@
         <v>128</v>
       </c>
       <c r="K43" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="n">

</xml_diff>